<commit_message>
Add gold_analysisETF.pyc and GDXJ.xlsx files
- Introduced a compiled Python file for gold analysis ETF functionality.
- Added a new Excel file containing user information for GDXJ.
</commit_message>
<xml_diff>
--- a/etf_gold_miners_uplift/rawGLD/GDX.xlsx
+++ b/etf_gold_miners_uplift/rawGLD/GDX.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GDX_asof_20260508" sheetId="1" r:id="R478a21afb71e4eaa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GDX_asof_20260513" sheetId="1" r:id="R272257d27e9d4a9f"/>
   </x:sheets>
 </x:workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="338">
-  <x:si>
-    <x:t>Daily Holdings (%)  05/08/2026</x:t>
+<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="334">
+  <x:si>
+    <x:t>Daily Holdings (%)  05/13/2026</x:t>
   </x:si>
   <x:si>
     <x:t/>
@@ -52,19 +52,19 @@
     <x:t>BBG000BPWXK1</x:t>
   </x:si>
   <x:si>
-    <x:t>27,699,963</x:t>
+    <x:t>27,690,875</x:t>
   </x:si>
   <x:si>
     <x:t>Stock</x:t>
   </x:si>
   <x:si>
-    <x:t>$3,227,322,689.13</x:t>
+    <x:t>$3,294,106,490.00</x:t>
   </x:si>
   <x:si>
     <x:t> -- </x:t>
   </x:si>
   <x:si>
-    <x:t>11.23%</x:t>
+    <x:t>11.22%</x:t>
   </x:si>
   <x:si>
     <x:t>AEM</x:t>
@@ -76,13 +76,13 @@
     <x:t>BBG000DLVDK3</x:t>
   </x:si>
   <x:si>
-    <x:t>16,568,097</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$3,201,122,021.37</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11.14%</x:t>
+    <x:t>16,562,661</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$3,245,784,676.17</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11.05%</x:t>
   </x:si>
   <x:si>
     <x:t>B</x:t>
@@ -94,13 +94,13 @@
     <x:t>BBG000BB07P9</x:t>
   </x:si>
   <x:si>
-    <x:t>52,077,005</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$2,246,081,225.65</x:t>
-  </x:si>
-  <x:si>
-    <x:t>7.82%</x:t>
+    <x:t>52,059,919</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$2,335,928,565.53</x:t>
+  </x:si>
+  <x:si>
+    <x:t>7.95%</x:t>
   </x:si>
   <x:si>
     <x:t>AU</x:t>
@@ -112,13 +112,13 @@
     <x:t>BBG01HGVLP51</x:t>
   </x:si>
   <x:si>
-    <x:t>14,549,337</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$1,557,215,539.11</x:t>
-  </x:si>
-  <x:si>
-    <x:t>5.42%</x:t>
+    <x:t>14,544,563</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$1,488,926,914.31</x:t>
+  </x:si>
+  <x:si>
+    <x:t>5.07%</x:t>
   </x:si>
   <x:si>
     <x:t>WPM</x:t>
@@ -130,10 +130,10 @@
     <x:t>BBG000PVRDL2</x:t>
   </x:si>
   <x:si>
-    <x:t>10,399,888</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$1,444,024,448.80</x:t>
+    <x:t>10,396,476</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$1,478,586,816.72</x:t>
   </x:si>
   <x:si>
     <x:t>5.03%</x:t>
@@ -148,13 +148,13 @@
     <x:t>BBG000RD3CL8</x:t>
   </x:si>
   <x:si>
-    <x:t>5,818,725</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$1,350,584,259.75</x:t>
-  </x:si>
-  <x:si>
-    <x:t>4.70%</x:t>
+    <x:t>5,816,815</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$1,400,630,883.85</x:t>
+  </x:si>
+  <x:si>
+    <x:t>4.77%</x:t>
   </x:si>
   <x:si>
     <x:t>KGC</x:t>
@@ -166,13 +166,13 @@
     <x:t>BBG000BB2DM7</x:t>
   </x:si>
   <x:si>
-    <x:t>42,737,690</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$1,346,664,611.90</x:t>
-  </x:si>
-  <x:si>
-    <x:t>4.69%</x:t>
+    <x:t>42,723,668</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$1,335,969,098.36</x:t>
+  </x:si>
+  <x:si>
+    <x:t>4.55%</x:t>
   </x:si>
   <x:si>
     <x:t>GFI</x:t>
@@ -184,13 +184,13 @@
     <x:t>BBG000KHT4K7</x:t>
   </x:si>
   <x:si>
-    <x:t>27,506,253</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$1,233,930,509.58</x:t>
-  </x:si>
-  <x:si>
-    <x:t>4.29%</x:t>
+    <x:t>27,497,229</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$1,231,325,914.62</x:t>
+  </x:si>
+  <x:si>
+    <x:t>4.19%</x:t>
   </x:si>
   <x:si>
     <x:t>PAAS</x:t>
@@ -202,13 +202,13 @@
     <x:t>BBG000C0RGY3</x:t>
   </x:si>
   <x:si>
-    <x:t>16,282,523</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$962,948,410.22</x:t>
-  </x:si>
-  <x:si>
-    <x:t>3.35%</x:t>
+    <x:t>16,277,181</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$1,036,205,342.46</x:t>
+  </x:si>
+  <x:si>
+    <x:t>3.53%</x:t>
   </x:si>
   <x:si>
     <x:t>NST AU</x:t>
@@ -220,13 +220,31 @@
     <x:t>BBG000C82NF9</x:t>
   </x:si>
   <x:si>
-    <x:t>50,021,929</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$767,037,072.04</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2.67%</x:t>
+    <x:t>50,005,517</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$780,613,235.57</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2.66%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CDE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Coeur Mining Inc</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BBG000BF8TF5</x:t>
+  </x:si>
+  <x:si>
+    <x:t>36,015,768</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$710,951,260.32</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2.42%</x:t>
   </x:si>
   <x:si>
     <x:t>AGI</x:t>
@@ -238,31 +256,13 @@
     <x:t>BBG009HT6BL4</x:t>
   </x:si>
   <x:si>
-    <x:t>16,014,331</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$694,701,678.78</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2.42%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CDE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Coeur Mining Inc</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BBG000BF8TF5</x:t>
-  </x:si>
-  <x:si>
-    <x:t>36,027,630</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$668,672,812.80</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2.33%</x:t>
+    <x:t>16,009,077</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$698,796,211.05</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2.38%</x:t>
   </x:si>
   <x:si>
     <x:t>RGLD</x:t>
@@ -274,10 +274,10 @@
     <x:t>BBG000BS5170</x:t>
   </x:si>
   <x:si>
-    <x:t>2,426,049</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$579,607,366.59</x:t>
+    <x:t>2,425,253</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$594,162,732.47</x:t>
   </x:si>
   <x:si>
     <x:t>2.02%</x:t>
@@ -292,13 +292,13 @@
     <x:t>BBG000LXSKQ0</x:t>
   </x:si>
   <x:si>
-    <x:t>8,482,533</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$500,877,133.10</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1.74%</x:t>
+    <x:t>8,479,753</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$524,447,539.08</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1.79%</x:t>
   </x:si>
   <x:si>
     <x:t>EDV LN</x:t>
@@ -310,13 +310,28 @@
     <x:t>BBG011DVVYT3</x:t>
   </x:si>
   <x:si>
-    <x:t>7,340,947</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$481,095,631.95</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1.67%</x:t>
+    <x:t>7,338,539</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$488,959,643.62</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1.66%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AG</x:t>
+  </x:si>
+  <x:si>
+    <x:t>First Majestic Silver Corp</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BBG000CH7WB8</x:t>
+  </x:si>
+  <x:si>
+    <x:t>20,362,657</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$488,296,514.86</x:t>
   </x:si>
   <x:si>
     <x:t>EVN AU</x:t>
@@ -328,13 +343,13 @@
     <x:t>BBG000NF2249</x:t>
   </x:si>
   <x:si>
-    <x:t>48,866,987</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$461,529,387.33</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1.61%</x:t>
+    <x:t>48,850,957</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$474,371,036.57</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1.62%</x:t>
   </x:si>
   <x:si>
     <x:t>EQX</x:t>
@@ -346,28 +361,10 @@
     <x:t>BBG004XB7MN9</x:t>
   </x:si>
   <x:si>
-    <x:t>31,497,413</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$450,098,031.77</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1.57%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AG</x:t>
-  </x:si>
-  <x:si>
-    <x:t>First Majestic Silver Corp</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BBG000CH7WB8</x:t>
-  </x:si>
-  <x:si>
-    <x:t>20,369,337</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$445,273,706.82</x:t>
+    <x:t>31,487,079</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$456,247,774.71</x:t>
   </x:si>
   <x:si>
     <x:t>1.55%</x:t>
@@ -382,13 +379,31 @@
     <x:t>BBG000VH0TC0</x:t>
   </x:si>
   <x:si>
-    <x:t>8,364,772</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$410,376,853.15</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1.43%</x:t>
+    <x:t>8,362,028</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$428,556,856.27</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1.46%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Hecla Mining Co</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BBG000BL5W86</x:t>
+  </x:si>
+  <x:si>
+    <x:t>18,865,165</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$397,111,723.25</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1.35%</x:t>
   </x:si>
   <x:si>
     <x:t>IAG</x:t>
@@ -400,31 +415,13 @@
     <x:t>BBG000LL9LQ5</x:t>
   </x:si>
   <x:si>
-    <x:t>19,539,806</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$365,394,372.20</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1.27%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Hecla Mining Co</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BBG000BL5W86</x:t>
-  </x:si>
-  <x:si>
-    <x:t>18,871,357</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$351,195,953.77</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1.22%</x:t>
+    <x:t>19,533,398</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$367,032,548.42</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1.25%</x:t>
   </x:si>
   <x:si>
     <x:t>LUG CN</x:t>
@@ -436,13 +433,49 @@
     <x:t>BBG000BZYV49</x:t>
   </x:si>
   <x:si>
-    <x:t>4,609,976</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$323,213,495.17</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1.12%</x:t>
+    <x:t>4,608,464</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$324,974,979.72</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1.11%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OGC CN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Oceanagold Corp</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BBG000RG1PM3</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9,400,991</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$322,684,239.95</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1.10%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EGO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Eldorado Gold Corp</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BBG000BN7277</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8,936,100</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$317,588,994.00</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1.08%</x:t>
   </x:si>
   <x:si>
     <x:t>HMY</x:t>
@@ -454,49 +487,49 @@
     <x:t>BBG000BX93G1</x:t>
   </x:si>
   <x:si>
-    <x:t>17,926,851</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$318,918,679.29</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1.11%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EGO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Eldorado Gold Corp</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BBG000BN7277</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8,939,032</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$305,267,942.80</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1.06%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>OGC CN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Oceanagold Corp</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BBG000RG1PM3</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9,404,077</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$299,823,213.10</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1.04%</x:t>
+    <x:t>17,920,969</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$314,513,005.95</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1.07%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BVN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Cia De Minas Buenaventura Saa</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BBG000GPXR82</x:t>
+  </x:si>
+  <x:si>
+    <x:t>7,860,830</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$302,406,130.10</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1.03%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BTG</x:t>
+  </x:si>
+  <x:si>
+    <x:t>B2gold Corp</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BBG000V9KFD5</x:t>
+  </x:si>
+  <x:si>
+    <x:t>51,060,090</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$273,682,082.40</x:t>
+  </x:si>
+  <x:si>
+    <x:t>0.93%</x:t>
   </x:si>
   <x:si>
     <x:t>1818 HK</x:t>
@@ -508,31 +541,10 @@
     <x:t>BBG000DQ77W9</x:t>
   </x:si>
   <x:si>
-    <x:t>74,526,000</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$285,315,167.81</x:t>
-  </x:si>
-  <x:si>
-    <x:t>0.99%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BVN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Cia De Minas Buenaventura Saa</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BBG000GPXR82</x:t>
-  </x:si>
-  <x:si>
-    <x:t>7,863,410</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$278,050,177.60</x:t>
-  </x:si>
-  <x:si>
-    <x:t>0.97%</x:t>
+    <x:t>74,502,000</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$273,265,899.79</x:t>
   </x:si>
   <x:si>
     <x:t>GMIN CN</x:t>
@@ -544,31 +556,10 @@
     <x:t>BBG01NT389N7</x:t>
   </x:si>
   <x:si>
-    <x:t>7,045,025</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$276,377,395.92</x:t>
-  </x:si>
-  <x:si>
-    <x:t>0.96%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BTG</x:t>
-  </x:si>
-  <x:si>
-    <x:t>B2gold Corp</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BBG000V9KFD5</x:t>
-  </x:si>
-  <x:si>
-    <x:t>51,076,848</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$270,707,294.40</x:t>
-  </x:si>
-  <x:si>
-    <x:t>0.94%</x:t>
+    <x:t>7,042,713</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$272,520,026.55</x:t>
   </x:si>
   <x:si>
     <x:t>SSRM</x:t>
@@ -580,13 +571,13 @@
     <x:t>BBG000C0RWX9</x:t>
   </x:si>
   <x:si>
-    <x:t>7,281,744</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$249,035,644.80</x:t>
-  </x:si>
-  <x:si>
-    <x:t>0.87%</x:t>
+    <x:t>7,279,354</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$252,957,551.50</x:t>
+  </x:si>
+  <x:si>
+    <x:t>0.86%</x:t>
   </x:si>
   <x:si>
     <x:t>DPM CN</x:t>
@@ -598,13 +589,13 @@
     <x:t>BBG000G9HTM6</x:t>
   </x:si>
   <x:si>
-    <x:t>6,953,010</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$240,518,993.21</x:t>
-  </x:si>
-  <x:si>
-    <x:t>0.84%</x:t>
+    <x:t>6,950,728</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$243,449,191.14</x:t>
+  </x:si>
+  <x:si>
+    <x:t>0.83%</x:t>
   </x:si>
   <x:si>
     <x:t>GGP AU</x:t>
@@ -616,13 +607,13 @@
     <x:t>BBG01V7BTM08</x:t>
   </x:si>
   <x:si>
-    <x:t>20,471,037</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$221,050,518.49</x:t>
-  </x:si>
-  <x:si>
-    <x:t>0.77%</x:t>
+    <x:t>20,464,321</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$219,550,632.83</x:t>
+  </x:si>
+  <x:si>
+    <x:t>0.75%</x:t>
   </x:si>
   <x:si>
     <x:t>DSV CN</x:t>
@@ -634,13 +625,13 @@
     <x:t>BBG000BS3HY7</x:t>
   </x:si>
   <x:si>
-    <x:t>28,184,494</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$199,273,903.97</x:t>
-  </x:si>
-  <x:si>
-    <x:t>0.69%</x:t>
+    <x:t>28,175,250</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$212,170,148.49</x:t>
+  </x:si>
+  <x:si>
+    <x:t>0.72%</x:t>
   </x:si>
   <x:si>
     <x:t>OR</x:t>
@@ -652,10 +643,10 @@
     <x:t>BBG006NTSJ78</x:t>
   </x:si>
   <x:si>
-    <x:t>5,022,677</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$192,971,250.34</x:t>
+    <x:t>5,021,029</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$196,824,336.80</x:t>
   </x:si>
   <x:si>
     <x:t>0.67%</x:t>
@@ -670,15 +661,33 @@
     <x:t>BBG000PMB297</x:t>
   </x:si>
   <x:si>
-    <x:t>74,235,746</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$188,977,347.89</x:t>
+    <x:t>74,211,392</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$192,421,532.53</x:t>
   </x:si>
   <x:si>
     <x:t>0.66%</x:t>
   </x:si>
   <x:si>
+    <x:t>KNT CN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>K92 Mining Inc</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BBG0018BVXB5</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8,524,392</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$175,096,964.35</x:t>
+  </x:si>
+  <x:si>
+    <x:t>0.60%</x:t>
+  </x:si>
+  <x:si>
     <x:t>ARMN</x:t>
   </x:si>
   <x:si>
@@ -688,13 +697,13 @@
     <x:t>BBG000K0VQL1</x:t>
   </x:si>
   <x:si>
-    <x:t>8,679,085</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$170,977,974.50</x:t>
-  </x:si>
-  <x:si>
-    <x:t>0.60%</x:t>
+    <x:t>8,676,237</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$171,008,631.27</x:t>
+  </x:si>
+  <x:si>
+    <x:t>0.58%</x:t>
   </x:si>
   <x:si>
     <x:t>TXG CN</x:t>
@@ -706,28 +715,61 @@
     <x:t>BBG000BSWRQ2</x:t>
   </x:si>
   <x:si>
-    <x:t>3,345,476</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$167,603,680.40</x:t>
-  </x:si>
-  <x:si>
-    <x:t>0.58%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KNT CN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>K92 Mining Inc</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BBG0018BVXB5</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8,527,190</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$165,673,255.42</x:t>
+    <x:t>3,344,378</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$168,921,044.30</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PRU AU</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Perseus Mining Ltd</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BBG000Q68231</x:t>
+  </x:si>
+  <x:si>
+    <x:t>41,094,292</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$168,478,291.16</x:t>
+  </x:si>
+  <x:si>
+    <x:t>0.57%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ARTG CN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Artemis Gold Inc</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BBG00PSSBKG8</x:t>
+  </x:si>
+  <x:si>
+    <x:t>6,100,920</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$159,996,398.85</x:t>
+  </x:si>
+  <x:si>
+    <x:t>0.54%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GMD AU</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Genesis Minerals Ltd</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BBG000J9HXY1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>33,184,782</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$159,725,207.50</x:t>
   </x:si>
   <x:si>
     <x:t>ORLA</x:t>
@@ -739,28 +781,79 @@
     <x:t>BBG00FZBZ5G6</x:t>
   </x:si>
   <x:si>
-    <x:t>10,948,518</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$164,665,710.72</x:t>
-  </x:si>
-  <x:si>
-    <x:t>0.57%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PRU AU</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Perseus Mining Ltd</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BBG000Q68231</x:t>
-  </x:si>
-  <x:si>
-    <x:t>41,107,776</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$164,369,875.26</x:t>
+    <x:t>10,944,926</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$159,577,021.08</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CGAU</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Centerra Gold Inc</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BBG000QWM2M7</x:t>
+  </x:si>
+  <x:si>
+    <x:t>7,981,049</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$150,682,205.12</x:t>
+  </x:si>
+  <x:si>
+    <x:t>0.51%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CMM AU</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Capricorn Metals Ltd</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BBG000C0X7Y6</x:t>
+  </x:si>
+  <x:si>
+    <x:t>14,304,258</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$145,946,898.17</x:t>
+  </x:si>
+  <x:si>
+    <x:t>0.50%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BRMS IJ</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Bumi Resources Minerals Tbk Pt</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BBG0018R2541</x:t>
+  </x:si>
+  <x:si>
+    <x:t>3,215,608,200</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$142,326,182.75</x:t>
+  </x:si>
+  <x:si>
+    <x:t>0.48%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EXK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Endeavour Silver Corp</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BBG000K2HB18</x:t>
+  </x:si>
+  <x:si>
+    <x:t>12,616,949</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$142,319,184.72</x:t>
   </x:si>
   <x:si>
     <x:t>AMMN IJ</x:t>
@@ -772,118 +865,10 @@
     <x:t>BBG01GVLB759</x:t>
   </x:si>
   <x:si>
-    <x:t>658,090,200</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$160,443,569.37</x:t>
-  </x:si>
-  <x:si>
-    <x:t>0.56%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ARTG CN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Artemis Gold Inc</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BBG00PSSBKG8</x:t>
-  </x:si>
-  <x:si>
-    <x:t>6,102,922</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$152,316,737.08</x:t>
-  </x:si>
-  <x:si>
-    <x:t>0.53%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GMD AU</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Genesis Minerals Ltd</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BBG000J9HXY1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>33,195,674</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$149,566,717.24</x:t>
-  </x:si>
-  <x:si>
-    <x:t>0.52%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CGAU</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Centerra Gold Inc</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BBG000QWM2M7</x:t>
-  </x:si>
-  <x:si>
-    <x:t>7,983,669</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$146,819,672.91</x:t>
-  </x:si>
-  <x:si>
-    <x:t>0.51%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CMM AU</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Capricorn Metals Ltd</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BBG000C0X7Y6</x:t>
-  </x:si>
-  <x:si>
-    <x:t>14,308,952</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$141,341,315.90</x:t>
-  </x:si>
-  <x:si>
-    <x:t>0.49%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BRMS IJ</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Bumi Resources Minerals Tbk Pt</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BBG0018R2541</x:t>
-  </x:si>
-  <x:si>
-    <x:t>3,216,664,000</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$140,228,860.14</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EXK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Endeavour Silver Corp</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BBG000K2HB18</x:t>
-  </x:si>
-  <x:si>
-    <x:t>12,621,087</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$126,589,502.61</x:t>
-  </x:si>
-  <x:si>
-    <x:t>0.44%</x:t>
+    <x:t>657,874,200</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$139,687,545.75</x:t>
   </x:si>
   <x:si>
     <x:t>WDO CN</x:t>
@@ -895,10 +880,13 @@
     <x:t>BBG000DKQDS3</x:t>
   </x:si>
   <x:si>
-    <x:t>6,145,385</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$126,085,650.90</x:t>
+    <x:t>6,143,369</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$138,785,584.47</x:t>
+  </x:si>
+  <x:si>
+    <x:t>0.47%</x:t>
   </x:si>
   <x:si>
     <x:t>WGX AU</x:t>
@@ -910,10 +898,10 @@
     <x:t>BBG000BG27F7</x:t>
   </x:si>
   <x:si>
-    <x:t>30,459,537</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$123,414,792.55</x:t>
+    <x:t>30,449,543</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$125,128,277.58</x:t>
   </x:si>
   <x:si>
     <x:t>0.43%</x:t>
@@ -928,13 +916,13 @@
     <x:t>BBG000LDZ482</x:t>
   </x:si>
   <x:si>
-    <x:t>11,088,470</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$119,311,937.20</x:t>
-  </x:si>
-  <x:si>
-    <x:t>0.42%</x:t>
+    <x:t>11,084,832</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$118,496,854.08</x:t>
+  </x:si>
+  <x:si>
+    <x:t>0.40%</x:t>
   </x:si>
   <x:si>
     <x:t>SA</x:t>
@@ -946,13 +934,10 @@
     <x:t>BBG000JYQX30</x:t>
   </x:si>
   <x:si>
-    <x:t>3,502,085</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$109,300,072.85</x:t>
-  </x:si>
-  <x:si>
-    <x:t>0.38%</x:t>
+    <x:t>3,500,939</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$116,441,231.14</x:t>
   </x:si>
   <x:si>
     <x:t>-USD CASH-</x:t>
@@ -961,27 +946,30 @@
     <x:t> </x:t>
   </x:si>
   <x:si>
-    <x:t>475,820</x:t>
+    <x:t>3,125,175</x:t>
   </x:si>
   <x:si>
     <x:t>Cash Bal</x:t>
   </x:si>
   <x:si>
-    <x:t>$475,819.78</x:t>
+    <x:t>$3,125,175.32</x:t>
+  </x:si>
+  <x:si>
+    <x:t>0.01%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>-IDR CASH-</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$.00</x:t>
   </x:si>
   <x:si>
     <x:t>0.00%</x:t>
   </x:si>
   <x:si>
-    <x:t>-IDR CASH-</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$.00</x:t>
-  </x:si>
-  <x:si>
     <x:t>-HKD CASH-</x:t>
   </x:si>
   <x:si>
@@ -997,7 +985,7 @@
     <x:t>424</x:t>
   </x:si>
   <x:si>
-    <x:t>$309.33</x:t>
+    <x:t>$309.03</x:t>
   </x:si>
   <x:si>
     <x:t>-AUD CASH-</x:t>
@@ -1006,7 +994,7 @@
     <x:t>940</x:t>
   </x:si>
   <x:si>
-    <x:t>$681.31</x:t>
+    <x:t>$682.53</x:t>
   </x:si>
   <x:si>
     <x:t>Other/Cash</x:t>
@@ -1015,7 +1003,7 @@
     <x:t>Cash</x:t>
   </x:si>
   <x:si>
-    <x:t>$9,151,047.18</x:t>
+    <x:t>$7,709,619.82</x:t>
   </x:si>
   <x:si>
     <x:t>0.03%</x:t>
@@ -1653,7 +1641,7 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="I19" s="1" t="s">
-        <x:v>108</x:v>
+        <x:v>102</x:v>
       </x:c>
     </x:row>
     <x:row r="20" spans="1:9" ht="15" customHeight="1">
@@ -1661,28 +1649,28 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="B20" s="1" t="s">
+        <x:v>108</x:v>
+      </x:c>
+      <x:c r="C20" s="1" t="s">
         <x:v>109</x:v>
       </x:c>
-      <x:c r="C20" s="1" t="s">
+      <x:c r="D20" s="1" t="s">
         <x:v>110</x:v>
       </x:c>
-      <x:c r="D20" s="1" t="s">
+      <x:c r="E20" s="1" t="s">
         <x:v>111</x:v>
       </x:c>
-      <x:c r="E20" s="1" t="s">
+      <x:c r="F20" s="1" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G20" s="1" t="s">
         <x:v>112</x:v>
       </x:c>
-      <x:c r="F20" s="1" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G20" s="1" t="s">
+      <x:c r="H20" s="1" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I20" s="1" t="s">
         <x:v>113</x:v>
-      </x:c>
-      <x:c r="H20" s="1" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I20" s="1" t="s">
-        <x:v>114</x:v>
       </x:c>
     </x:row>
     <x:row r="21" spans="1:9" ht="15" customHeight="1">
@@ -1690,28 +1678,28 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="B21" s="1" t="s">
+        <x:v>114</x:v>
+      </x:c>
+      <x:c r="C21" s="1" t="s">
         <x:v>115</x:v>
       </x:c>
-      <x:c r="C21" s="1" t="s">
+      <x:c r="D21" s="1" t="s">
         <x:v>116</x:v>
       </x:c>
-      <x:c r="D21" s="1" t="s">
+      <x:c r="E21" s="1" t="s">
         <x:v>117</x:v>
       </x:c>
-      <x:c r="E21" s="1" t="s">
+      <x:c r="F21" s="1" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G21" s="1" t="s">
         <x:v>118</x:v>
       </x:c>
-      <x:c r="F21" s="1" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G21" s="1" t="s">
+      <x:c r="H21" s="1" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I21" s="1" t="s">
         <x:v>119</x:v>
-      </x:c>
-      <x:c r="H21" s="1" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I21" s="1" t="s">
-        <x:v>120</x:v>
       </x:c>
     </x:row>
     <x:row r="22" spans="1:9" ht="15" customHeight="1">
@@ -1719,28 +1707,28 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="B22" s="1" t="s">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="C22" s="1" t="s">
         <x:v>121</x:v>
       </x:c>
-      <x:c r="C22" s="1" t="s">
+      <x:c r="D22" s="1" t="s">
         <x:v>122</x:v>
       </x:c>
-      <x:c r="D22" s="1" t="s">
+      <x:c r="E22" s="1" t="s">
         <x:v>123</x:v>
       </x:c>
-      <x:c r="E22" s="1" t="s">
+      <x:c r="F22" s="1" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G22" s="1" t="s">
         <x:v>124</x:v>
       </x:c>
-      <x:c r="F22" s="1" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G22" s="1" t="s">
+      <x:c r="H22" s="1" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I22" s="1" t="s">
         <x:v>125</x:v>
-      </x:c>
-      <x:c r="H22" s="1" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I22" s="1" t="s">
-        <x:v>126</x:v>
       </x:c>
     </x:row>
     <x:row r="23" spans="1:9" ht="15" customHeight="1">
@@ -1748,28 +1736,28 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="B23" s="1" t="s">
+        <x:v>126</x:v>
+      </x:c>
+      <x:c r="C23" s="1" t="s">
         <x:v>127</x:v>
       </x:c>
-      <x:c r="C23" s="1" t="s">
+      <x:c r="D23" s="1" t="s">
         <x:v>128</x:v>
       </x:c>
-      <x:c r="D23" s="1" t="s">
+      <x:c r="E23" s="1" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="E23" s="1" t="s">
+      <x:c r="F23" s="1" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G23" s="1" t="s">
         <x:v>130</x:v>
       </x:c>
-      <x:c r="F23" s="1" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G23" s="1" t="s">
+      <x:c r="H23" s="1" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I23" s="1" t="s">
         <x:v>131</x:v>
-      </x:c>
-      <x:c r="H23" s="1" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I23" s="1" t="s">
-        <x:v>132</x:v>
       </x:c>
     </x:row>
     <x:row r="24" spans="1:9" ht="15" customHeight="1">
@@ -1777,28 +1765,28 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="B24" s="1" t="s">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="C24" s="1" t="s">
         <x:v>133</x:v>
       </x:c>
-      <x:c r="C24" s="1" t="s">
+      <x:c r="D24" s="1" t="s">
         <x:v>134</x:v>
       </x:c>
-      <x:c r="D24" s="1" t="s">
+      <x:c r="E24" s="1" t="s">
         <x:v>135</x:v>
       </x:c>
-      <x:c r="E24" s="1" t="s">
+      <x:c r="F24" s="1" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G24" s="1" t="s">
         <x:v>136</x:v>
       </x:c>
-      <x:c r="F24" s="1" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G24" s="1" t="s">
+      <x:c r="H24" s="1" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I24" s="1" t="s">
         <x:v>137</x:v>
-      </x:c>
-      <x:c r="H24" s="1" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I24" s="1" t="s">
-        <x:v>138</x:v>
       </x:c>
     </x:row>
     <x:row r="25" spans="1:9" ht="15" customHeight="1">
@@ -1806,28 +1794,28 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B25" s="1" t="s">
+        <x:v>138</x:v>
+      </x:c>
+      <x:c r="C25" s="1" t="s">
         <x:v>139</x:v>
       </x:c>
-      <x:c r="C25" s="1" t="s">
+      <x:c r="D25" s="1" t="s">
         <x:v>140</x:v>
       </x:c>
-      <x:c r="D25" s="1" t="s">
+      <x:c r="E25" s="1" t="s">
         <x:v>141</x:v>
       </x:c>
-      <x:c r="E25" s="1" t="s">
+      <x:c r="F25" s="1" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G25" s="1" t="s">
         <x:v>142</x:v>
       </x:c>
-      <x:c r="F25" s="1" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G25" s="1" t="s">
+      <x:c r="H25" s="1" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I25" s="1" t="s">
         <x:v>143</x:v>
-      </x:c>
-      <x:c r="H25" s="1" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I25" s="1" t="s">
-        <x:v>144</x:v>
       </x:c>
     </x:row>
     <x:row r="26" spans="1:9" ht="15" customHeight="1">
@@ -1835,28 +1823,28 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="B26" s="1" t="s">
+        <x:v>144</x:v>
+      </x:c>
+      <x:c r="C26" s="1" t="s">
         <x:v>145</x:v>
       </x:c>
-      <x:c r="C26" s="1" t="s">
+      <x:c r="D26" s="1" t="s">
         <x:v>146</x:v>
       </x:c>
-      <x:c r="D26" s="1" t="s">
+      <x:c r="E26" s="1" t="s">
         <x:v>147</x:v>
       </x:c>
-      <x:c r="E26" s="1" t="s">
+      <x:c r="F26" s="1" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G26" s="1" t="s">
         <x:v>148</x:v>
       </x:c>
-      <x:c r="F26" s="1" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G26" s="1" t="s">
+      <x:c r="H26" s="1" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I26" s="1" t="s">
         <x:v>149</x:v>
-      </x:c>
-      <x:c r="H26" s="1" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I26" s="1" t="s">
-        <x:v>150</x:v>
       </x:c>
     </x:row>
     <x:row r="27" spans="1:9" ht="15" customHeight="1">
@@ -1864,28 +1852,28 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="B27" s="1" t="s">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="C27" s="1" t="s">
         <x:v>151</x:v>
       </x:c>
-      <x:c r="C27" s="1" t="s">
+      <x:c r="D27" s="1" t="s">
         <x:v>152</x:v>
       </x:c>
-      <x:c r="D27" s="1" t="s">
+      <x:c r="E27" s="1" t="s">
         <x:v>153</x:v>
       </x:c>
-      <x:c r="E27" s="1" t="s">
+      <x:c r="F27" s="1" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G27" s="1" t="s">
         <x:v>154</x:v>
       </x:c>
-      <x:c r="F27" s="1" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G27" s="1" t="s">
+      <x:c r="H27" s="1" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I27" s="1" t="s">
         <x:v>155</x:v>
-      </x:c>
-      <x:c r="H27" s="1" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I27" s="1" t="s">
-        <x:v>156</x:v>
       </x:c>
     </x:row>
     <x:row r="28" spans="1:9" ht="15" customHeight="1">
@@ -1893,28 +1881,28 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="B28" s="1" t="s">
+        <x:v>156</x:v>
+      </x:c>
+      <x:c r="C28" s="1" t="s">
         <x:v>157</x:v>
       </x:c>
-      <x:c r="C28" s="1" t="s">
+      <x:c r="D28" s="1" t="s">
         <x:v>158</x:v>
       </x:c>
-      <x:c r="D28" s="1" t="s">
+      <x:c r="E28" s="1" t="s">
         <x:v>159</x:v>
       </x:c>
-      <x:c r="E28" s="1" t="s">
+      <x:c r="F28" s="1" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G28" s="1" t="s">
         <x:v>160</x:v>
       </x:c>
-      <x:c r="F28" s="1" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G28" s="1" t="s">
+      <x:c r="H28" s="1" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I28" s="1" t="s">
         <x:v>161</x:v>
-      </x:c>
-      <x:c r="H28" s="1" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I28" s="1" t="s">
-        <x:v>162</x:v>
       </x:c>
     </x:row>
     <x:row r="29" spans="1:9" ht="15" customHeight="1">
@@ -1922,28 +1910,28 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="B29" s="1" t="s">
+        <x:v>162</x:v>
+      </x:c>
+      <x:c r="C29" s="1" t="s">
         <x:v>163</x:v>
       </x:c>
-      <x:c r="C29" s="1" t="s">
+      <x:c r="D29" s="1" t="s">
         <x:v>164</x:v>
       </x:c>
-      <x:c r="D29" s="1" t="s">
+      <x:c r="E29" s="1" t="s">
         <x:v>165</x:v>
       </x:c>
-      <x:c r="E29" s="1" t="s">
+      <x:c r="F29" s="1" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G29" s="1" t="s">
         <x:v>166</x:v>
       </x:c>
-      <x:c r="F29" s="1" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G29" s="1" t="s">
+      <x:c r="H29" s="1" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I29" s="1" t="s">
         <x:v>167</x:v>
-      </x:c>
-      <x:c r="H29" s="1" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I29" s="1" t="s">
-        <x:v>168</x:v>
       </x:c>
     </x:row>
     <x:row r="30" spans="1:9" ht="15" customHeight="1">
@@ -1951,28 +1939,28 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="B30" s="1" t="s">
+        <x:v>168</x:v>
+      </x:c>
+      <x:c r="C30" s="1" t="s">
         <x:v>169</x:v>
       </x:c>
-      <x:c r="C30" s="1" t="s">
+      <x:c r="D30" s="1" t="s">
         <x:v>170</x:v>
       </x:c>
-      <x:c r="D30" s="1" t="s">
+      <x:c r="E30" s="1" t="s">
         <x:v>171</x:v>
       </x:c>
-      <x:c r="E30" s="1" t="s">
+      <x:c r="F30" s="1" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G30" s="1" t="s">
         <x:v>172</x:v>
       </x:c>
-      <x:c r="F30" s="1" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G30" s="1" t="s">
+      <x:c r="H30" s="1" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I30" s="1" t="s">
         <x:v>173</x:v>
-      </x:c>
-      <x:c r="H30" s="1" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I30" s="1" t="s">
-        <x:v>174</x:v>
       </x:c>
     </x:row>
     <x:row r="31" spans="1:9" ht="15" customHeight="1">
@@ -1980,28 +1968,28 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="B31" s="1" t="s">
+        <x:v>174</x:v>
+      </x:c>
+      <x:c r="C31" s="1" t="s">
         <x:v>175</x:v>
       </x:c>
-      <x:c r="C31" s="1" t="s">
+      <x:c r="D31" s="1" t="s">
         <x:v>176</x:v>
       </x:c>
-      <x:c r="D31" s="1" t="s">
+      <x:c r="E31" s="1" t="s">
         <x:v>177</x:v>
       </x:c>
-      <x:c r="E31" s="1" t="s">
+      <x:c r="F31" s="1" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G31" s="1" t="s">
         <x:v>178</x:v>
       </x:c>
-      <x:c r="F31" s="1" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G31" s="1" t="s">
-        <x:v>179</x:v>
-      </x:c>
       <x:c r="H31" s="1" t="s">
         <x:v>17</x:v>
       </x:c>
       <x:c r="I31" s="1" t="s">
-        <x:v>180</x:v>
+        <x:v>173</x:v>
       </x:c>
     </x:row>
     <x:row r="32" spans="1:9" ht="15" customHeight="1">
@@ -2009,28 +1997,28 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="B32" s="1" t="s">
+        <x:v>179</x:v>
+      </x:c>
+      <x:c r="C32" s="1" t="s">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="D32" s="1" t="s">
         <x:v>181</x:v>
       </x:c>
-      <x:c r="C32" s="1" t="s">
+      <x:c r="E32" s="1" t="s">
         <x:v>182</x:v>
       </x:c>
-      <x:c r="D32" s="1" t="s">
+      <x:c r="F32" s="1" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G32" s="1" t="s">
         <x:v>183</x:v>
       </x:c>
-      <x:c r="E32" s="1" t="s">
-        <x:v>184</x:v>
-      </x:c>
-      <x:c r="F32" s="1" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G32" s="1" t="s">
-        <x:v>185</x:v>
-      </x:c>
       <x:c r="H32" s="1" t="s">
         <x:v>17</x:v>
       </x:c>
       <x:c r="I32" s="1" t="s">
-        <x:v>186</x:v>
+        <x:v>173</x:v>
       </x:c>
     </x:row>
     <x:row r="33" spans="1:9" ht="15" customHeight="1">
@@ -2038,28 +2026,28 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="B33" s="1" t="s">
+        <x:v>184</x:v>
+      </x:c>
+      <x:c r="C33" s="1" t="s">
+        <x:v>185</x:v>
+      </x:c>
+      <x:c r="D33" s="1" t="s">
+        <x:v>186</x:v>
+      </x:c>
+      <x:c r="E33" s="1" t="s">
         <x:v>187</x:v>
       </x:c>
-      <x:c r="C33" s="1" t="s">
+      <x:c r="F33" s="1" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G33" s="1" t="s">
         <x:v>188</x:v>
       </x:c>
-      <x:c r="D33" s="1" t="s">
+      <x:c r="H33" s="1" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I33" s="1" t="s">
         <x:v>189</x:v>
-      </x:c>
-      <x:c r="E33" s="1" t="s">
-        <x:v>190</x:v>
-      </x:c>
-      <x:c r="F33" s="1" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G33" s="1" t="s">
-        <x:v>191</x:v>
-      </x:c>
-      <x:c r="H33" s="1" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I33" s="1" t="s">
-        <x:v>192</x:v>
       </x:c>
     </x:row>
     <x:row r="34" spans="1:9" ht="15" customHeight="1">
@@ -2067,28 +2055,28 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="B34" s="1" t="s">
+        <x:v>190</x:v>
+      </x:c>
+      <x:c r="C34" s="1" t="s">
+        <x:v>191</x:v>
+      </x:c>
+      <x:c r="D34" s="1" t="s">
+        <x:v>192</x:v>
+      </x:c>
+      <x:c r="E34" s="1" t="s">
         <x:v>193</x:v>
       </x:c>
-      <x:c r="C34" s="1" t="s">
+      <x:c r="F34" s="1" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G34" s="1" t="s">
         <x:v>194</x:v>
       </x:c>
-      <x:c r="D34" s="1" t="s">
+      <x:c r="H34" s="1" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I34" s="1" t="s">
         <x:v>195</x:v>
-      </x:c>
-      <x:c r="E34" s="1" t="s">
-        <x:v>196</x:v>
-      </x:c>
-      <x:c r="F34" s="1" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G34" s="1" t="s">
-        <x:v>197</x:v>
-      </x:c>
-      <x:c r="H34" s="1" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I34" s="1" t="s">
-        <x:v>198</x:v>
       </x:c>
     </x:row>
     <x:row r="35" spans="1:9" ht="15" customHeight="1">
@@ -2096,28 +2084,28 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="B35" s="1" t="s">
+        <x:v>196</x:v>
+      </x:c>
+      <x:c r="C35" s="1" t="s">
+        <x:v>197</x:v>
+      </x:c>
+      <x:c r="D35" s="1" t="s">
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="E35" s="1" t="s">
         <x:v>199</x:v>
       </x:c>
-      <x:c r="C35" s="1" t="s">
+      <x:c r="F35" s="1" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G35" s="1" t="s">
         <x:v>200</x:v>
       </x:c>
-      <x:c r="D35" s="1" t="s">
+      <x:c r="H35" s="1" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I35" s="1" t="s">
         <x:v>201</x:v>
-      </x:c>
-      <x:c r="E35" s="1" t="s">
-        <x:v>202</x:v>
-      </x:c>
-      <x:c r="F35" s="1" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G35" s="1" t="s">
-        <x:v>203</x:v>
-      </x:c>
-      <x:c r="H35" s="1" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I35" s="1" t="s">
-        <x:v>204</x:v>
       </x:c>
     </x:row>
     <x:row r="36" spans="1:9" ht="15" customHeight="1">
@@ -2125,28 +2113,28 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="B36" s="1" t="s">
+        <x:v>202</x:v>
+      </x:c>
+      <x:c r="C36" s="1" t="s">
+        <x:v>203</x:v>
+      </x:c>
+      <x:c r="D36" s="1" t="s">
+        <x:v>204</x:v>
+      </x:c>
+      <x:c r="E36" s="1" t="s">
         <x:v>205</x:v>
       </x:c>
-      <x:c r="C36" s="1" t="s">
+      <x:c r="F36" s="1" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G36" s="1" t="s">
         <x:v>206</x:v>
       </x:c>
-      <x:c r="D36" s="1" t="s">
+      <x:c r="H36" s="1" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I36" s="1" t="s">
         <x:v>207</x:v>
-      </x:c>
-      <x:c r="E36" s="1" t="s">
-        <x:v>208</x:v>
-      </x:c>
-      <x:c r="F36" s="1" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G36" s="1" t="s">
-        <x:v>209</x:v>
-      </x:c>
-      <x:c r="H36" s="1" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I36" s="1" t="s">
-        <x:v>210</x:v>
       </x:c>
     </x:row>
     <x:row r="37" spans="1:9" ht="15" customHeight="1">
@@ -2154,28 +2142,28 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="B37" s="1" t="s">
+        <x:v>208</x:v>
+      </x:c>
+      <x:c r="C37" s="1" t="s">
+        <x:v>209</x:v>
+      </x:c>
+      <x:c r="D37" s="1" t="s">
+        <x:v>210</x:v>
+      </x:c>
+      <x:c r="E37" s="1" t="s">
         <x:v>211</x:v>
       </x:c>
-      <x:c r="C37" s="1" t="s">
+      <x:c r="F37" s="1" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G37" s="1" t="s">
         <x:v>212</x:v>
       </x:c>
-      <x:c r="D37" s="1" t="s">
+      <x:c r="H37" s="1" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I37" s="1" t="s">
         <x:v>213</x:v>
-      </x:c>
-      <x:c r="E37" s="1" t="s">
-        <x:v>214</x:v>
-      </x:c>
-      <x:c r="F37" s="1" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G37" s="1" t="s">
-        <x:v>215</x:v>
-      </x:c>
-      <x:c r="H37" s="1" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I37" s="1" t="s">
-        <x:v>216</x:v>
       </x:c>
     </x:row>
     <x:row r="38" spans="1:9" ht="15" customHeight="1">
@@ -2183,28 +2171,28 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="B38" s="1" t="s">
+        <x:v>214</x:v>
+      </x:c>
+      <x:c r="C38" s="1" t="s">
+        <x:v>215</x:v>
+      </x:c>
+      <x:c r="D38" s="1" t="s">
+        <x:v>216</x:v>
+      </x:c>
+      <x:c r="E38" s="1" t="s">
         <x:v>217</x:v>
       </x:c>
-      <x:c r="C38" s="1" t="s">
+      <x:c r="F38" s="1" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G38" s="1" t="s">
         <x:v>218</x:v>
       </x:c>
-      <x:c r="D38" s="1" t="s">
+      <x:c r="H38" s="1" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I38" s="1" t="s">
         <x:v>219</x:v>
-      </x:c>
-      <x:c r="E38" s="1" t="s">
-        <x:v>220</x:v>
-      </x:c>
-      <x:c r="F38" s="1" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G38" s="1" t="s">
-        <x:v>221</x:v>
-      </x:c>
-      <x:c r="H38" s="1" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I38" s="1" t="s">
-        <x:v>222</x:v>
       </x:c>
     </x:row>
     <x:row r="39" spans="1:9" ht="15" customHeight="1">
@@ -2212,28 +2200,28 @@
         <x:v>36</x:v>
       </x:c>
       <x:c r="B39" s="1" t="s">
+        <x:v>220</x:v>
+      </x:c>
+      <x:c r="C39" s="1" t="s">
+        <x:v>221</x:v>
+      </x:c>
+      <x:c r="D39" s="1" t="s">
+        <x:v>222</x:v>
+      </x:c>
+      <x:c r="E39" s="1" t="s">
         <x:v>223</x:v>
       </x:c>
-      <x:c r="C39" s="1" t="s">
+      <x:c r="F39" s="1" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G39" s="1" t="s">
         <x:v>224</x:v>
       </x:c>
-      <x:c r="D39" s="1" t="s">
+      <x:c r="H39" s="1" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I39" s="1" t="s">
         <x:v>225</x:v>
-      </x:c>
-      <x:c r="E39" s="1" t="s">
-        <x:v>226</x:v>
-      </x:c>
-      <x:c r="F39" s="1" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G39" s="1" t="s">
-        <x:v>227</x:v>
-      </x:c>
-      <x:c r="H39" s="1" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I39" s="1" t="s">
-        <x:v>228</x:v>
       </x:c>
     </x:row>
     <x:row r="40" spans="1:9" ht="15" customHeight="1">
@@ -2241,28 +2229,28 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="B40" s="1" t="s">
+        <x:v>226</x:v>
+      </x:c>
+      <x:c r="C40" s="1" t="s">
+        <x:v>227</x:v>
+      </x:c>
+      <x:c r="D40" s="1" t="s">
+        <x:v>228</x:v>
+      </x:c>
+      <x:c r="E40" s="1" t="s">
         <x:v>229</x:v>
       </x:c>
-      <x:c r="C40" s="1" t="s">
+      <x:c r="F40" s="1" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G40" s="1" t="s">
         <x:v>230</x:v>
       </x:c>
-      <x:c r="D40" s="1" t="s">
+      <x:c r="H40" s="1" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I40" s="1" t="s">
         <x:v>231</x:v>
-      </x:c>
-      <x:c r="E40" s="1" t="s">
-        <x:v>232</x:v>
-      </x:c>
-      <x:c r="F40" s="1" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G40" s="1" t="s">
-        <x:v>233</x:v>
-      </x:c>
-      <x:c r="H40" s="1" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I40" s="1" t="s">
-        <x:v>234</x:v>
       </x:c>
     </x:row>
     <x:row r="41" spans="1:9" ht="15" customHeight="1">
@@ -2270,28 +2258,28 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="B41" s="1" t="s">
+        <x:v>232</x:v>
+      </x:c>
+      <x:c r="C41" s="1" t="s">
+        <x:v>233</x:v>
+      </x:c>
+      <x:c r="D41" s="1" t="s">
+        <x:v>234</x:v>
+      </x:c>
+      <x:c r="E41" s="1" t="s">
         <x:v>235</x:v>
       </x:c>
-      <x:c r="C41" s="1" t="s">
+      <x:c r="F41" s="1" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G41" s="1" t="s">
         <x:v>236</x:v>
       </x:c>
-      <x:c r="D41" s="1" t="s">
-        <x:v>237</x:v>
-      </x:c>
-      <x:c r="E41" s="1" t="s">
-        <x:v>238</x:v>
-      </x:c>
-      <x:c r="F41" s="1" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G41" s="1" t="s">
-        <x:v>239</x:v>
-      </x:c>
       <x:c r="H41" s="1" t="s">
         <x:v>17</x:v>
       </x:c>
       <x:c r="I41" s="1" t="s">
-        <x:v>234</x:v>
+        <x:v>231</x:v>
       </x:c>
     </x:row>
     <x:row r="42" spans="1:9" ht="15" customHeight="1">
@@ -2299,28 +2287,28 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="B42" s="1" t="s">
+        <x:v>237</x:v>
+      </x:c>
+      <x:c r="C42" s="1" t="s">
+        <x:v>238</x:v>
+      </x:c>
+      <x:c r="D42" s="1" t="s">
+        <x:v>239</x:v>
+      </x:c>
+      <x:c r="E42" s="1" t="s">
         <x:v>240</x:v>
       </x:c>
-      <x:c r="C42" s="1" t="s">
+      <x:c r="F42" s="1" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G42" s="1" t="s">
         <x:v>241</x:v>
       </x:c>
-      <x:c r="D42" s="1" t="s">
+      <x:c r="H42" s="1" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I42" s="1" t="s">
         <x:v>242</x:v>
-      </x:c>
-      <x:c r="E42" s="1" t="s">
-        <x:v>243</x:v>
-      </x:c>
-      <x:c r="F42" s="1" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G42" s="1" t="s">
-        <x:v>244</x:v>
-      </x:c>
-      <x:c r="H42" s="1" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I42" s="1" t="s">
-        <x:v>245</x:v>
       </x:c>
     </x:row>
     <x:row r="43" spans="1:9" ht="15" customHeight="1">
@@ -2328,28 +2316,28 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="B43" s="1" t="s">
+        <x:v>243</x:v>
+      </x:c>
+      <x:c r="C43" s="1" t="s">
+        <x:v>244</x:v>
+      </x:c>
+      <x:c r="D43" s="1" t="s">
+        <x:v>245</x:v>
+      </x:c>
+      <x:c r="E43" s="1" t="s">
         <x:v>246</x:v>
       </x:c>
-      <x:c r="C43" s="1" t="s">
+      <x:c r="F43" s="1" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G43" s="1" t="s">
         <x:v>247</x:v>
       </x:c>
-      <x:c r="D43" s="1" t="s">
+      <x:c r="H43" s="1" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I43" s="1" t="s">
         <x:v>248</x:v>
-      </x:c>
-      <x:c r="E43" s="1" t="s">
-        <x:v>249</x:v>
-      </x:c>
-      <x:c r="F43" s="1" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G43" s="1" t="s">
-        <x:v>250</x:v>
-      </x:c>
-      <x:c r="H43" s="1" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I43" s="1" t="s">
-        <x:v>245</x:v>
       </x:c>
     </x:row>
     <x:row r="44" spans="1:9" ht="15" customHeight="1">
@@ -2357,28 +2345,28 @@
         <x:v>41</x:v>
       </x:c>
       <x:c r="B44" s="1" t="s">
+        <x:v>249</x:v>
+      </x:c>
+      <x:c r="C44" s="1" t="s">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="D44" s="1" t="s">
         <x:v>251</x:v>
       </x:c>
-      <x:c r="C44" s="1" t="s">
+      <x:c r="E44" s="1" t="s">
         <x:v>252</x:v>
       </x:c>
-      <x:c r="D44" s="1" t="s">
+      <x:c r="F44" s="1" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G44" s="1" t="s">
         <x:v>253</x:v>
       </x:c>
-      <x:c r="E44" s="1" t="s">
-        <x:v>254</x:v>
-      </x:c>
-      <x:c r="F44" s="1" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G44" s="1" t="s">
-        <x:v>255</x:v>
-      </x:c>
       <x:c r="H44" s="1" t="s">
         <x:v>17</x:v>
       </x:c>
       <x:c r="I44" s="1" t="s">
-        <x:v>256</x:v>
+        <x:v>248</x:v>
       </x:c>
     </x:row>
     <x:row r="45" spans="1:9" ht="15" customHeight="1">
@@ -2386,28 +2374,28 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="B45" s="1" t="s">
+        <x:v>254</x:v>
+      </x:c>
+      <x:c r="C45" s="1" t="s">
+        <x:v>255</x:v>
+      </x:c>
+      <x:c r="D45" s="1" t="s">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="E45" s="1" t="s">
         <x:v>257</x:v>
       </x:c>
-      <x:c r="C45" s="1" t="s">
+      <x:c r="F45" s="1" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G45" s="1" t="s">
         <x:v>258</x:v>
       </x:c>
-      <x:c r="D45" s="1" t="s">
-        <x:v>259</x:v>
-      </x:c>
-      <x:c r="E45" s="1" t="s">
-        <x:v>260</x:v>
-      </x:c>
-      <x:c r="F45" s="1" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G45" s="1" t="s">
-        <x:v>261</x:v>
-      </x:c>
       <x:c r="H45" s="1" t="s">
         <x:v>17</x:v>
       </x:c>
       <x:c r="I45" s="1" t="s">
-        <x:v>262</x:v>
+        <x:v>248</x:v>
       </x:c>
     </x:row>
     <x:row r="46" spans="1:9" ht="15" customHeight="1">
@@ -2415,28 +2403,28 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="B46" s="1" t="s">
+        <x:v>259</x:v>
+      </x:c>
+      <x:c r="C46" s="1" t="s">
+        <x:v>260</x:v>
+      </x:c>
+      <x:c r="D46" s="1" t="s">
+        <x:v>261</x:v>
+      </x:c>
+      <x:c r="E46" s="1" t="s">
+        <x:v>262</x:v>
+      </x:c>
+      <x:c r="F46" s="1" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G46" s="1" t="s">
         <x:v>263</x:v>
       </x:c>
-      <x:c r="C46" s="1" t="s">
+      <x:c r="H46" s="1" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I46" s="1" t="s">
         <x:v>264</x:v>
-      </x:c>
-      <x:c r="D46" s="1" t="s">
-        <x:v>265</x:v>
-      </x:c>
-      <x:c r="E46" s="1" t="s">
-        <x:v>266</x:v>
-      </x:c>
-      <x:c r="F46" s="1" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G46" s="1" t="s">
-        <x:v>267</x:v>
-      </x:c>
-      <x:c r="H46" s="1" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I46" s="1" t="s">
-        <x:v>268</x:v>
       </x:c>
     </x:row>
     <x:row r="47" spans="1:9" ht="15" customHeight="1">
@@ -2444,28 +2432,28 @@
         <x:v>44</x:v>
       </x:c>
       <x:c r="B47" s="1" t="s">
+        <x:v>265</x:v>
+      </x:c>
+      <x:c r="C47" s="1" t="s">
+        <x:v>266</x:v>
+      </x:c>
+      <x:c r="D47" s="1" t="s">
+        <x:v>267</x:v>
+      </x:c>
+      <x:c r="E47" s="1" t="s">
+        <x:v>268</x:v>
+      </x:c>
+      <x:c r="F47" s="1" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G47" s="1" t="s">
         <x:v>269</x:v>
       </x:c>
-      <x:c r="C47" s="1" t="s">
+      <x:c r="H47" s="1" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I47" s="1" t="s">
         <x:v>270</x:v>
-      </x:c>
-      <x:c r="D47" s="1" t="s">
-        <x:v>271</x:v>
-      </x:c>
-      <x:c r="E47" s="1" t="s">
-        <x:v>272</x:v>
-      </x:c>
-      <x:c r="F47" s="1" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G47" s="1" t="s">
-        <x:v>273</x:v>
-      </x:c>
-      <x:c r="H47" s="1" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I47" s="1" t="s">
-        <x:v>274</x:v>
       </x:c>
     </x:row>
     <x:row r="48" spans="1:9" ht="15" customHeight="1">
@@ -2473,28 +2461,28 @@
         <x:v>45</x:v>
       </x:c>
       <x:c r="B48" s="1" t="s">
+        <x:v>271</x:v>
+      </x:c>
+      <x:c r="C48" s="1" t="s">
+        <x:v>272</x:v>
+      </x:c>
+      <x:c r="D48" s="1" t="s">
+        <x:v>273</x:v>
+      </x:c>
+      <x:c r="E48" s="1" t="s">
+        <x:v>274</x:v>
+      </x:c>
+      <x:c r="F48" s="1" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G48" s="1" t="s">
         <x:v>275</x:v>
       </x:c>
-      <x:c r="C48" s="1" t="s">
+      <x:c r="H48" s="1" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I48" s="1" t="s">
         <x:v>276</x:v>
-      </x:c>
-      <x:c r="D48" s="1" t="s">
-        <x:v>277</x:v>
-      </x:c>
-      <x:c r="E48" s="1" t="s">
-        <x:v>278</x:v>
-      </x:c>
-      <x:c r="F48" s="1" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G48" s="1" t="s">
-        <x:v>279</x:v>
-      </x:c>
-      <x:c r="H48" s="1" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I48" s="1" t="s">
-        <x:v>280</x:v>
       </x:c>
     </x:row>
     <x:row r="49" spans="1:9" ht="15" customHeight="1">
@@ -2502,28 +2490,28 @@
         <x:v>46</x:v>
       </x:c>
       <x:c r="B49" s="1" t="s">
+        <x:v>277</x:v>
+      </x:c>
+      <x:c r="C49" s="1" t="s">
+        <x:v>278</x:v>
+      </x:c>
+      <x:c r="D49" s="1" t="s">
+        <x:v>279</x:v>
+      </x:c>
+      <x:c r="E49" s="1" t="s">
+        <x:v>280</x:v>
+      </x:c>
+      <x:c r="F49" s="1" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G49" s="1" t="s">
         <x:v>281</x:v>
       </x:c>
-      <x:c r="C49" s="1" t="s">
-        <x:v>282</x:v>
-      </x:c>
-      <x:c r="D49" s="1" t="s">
-        <x:v>283</x:v>
-      </x:c>
-      <x:c r="E49" s="1" t="s">
-        <x:v>284</x:v>
-      </x:c>
-      <x:c r="F49" s="1" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G49" s="1" t="s">
-        <x:v>285</x:v>
-      </x:c>
       <x:c r="H49" s="1" t="s">
         <x:v>17</x:v>
       </x:c>
       <x:c r="I49" s="1" t="s">
-        <x:v>280</x:v>
+        <x:v>276</x:v>
       </x:c>
     </x:row>
     <x:row r="50" spans="1:9" ht="15" customHeight="1">
@@ -2531,28 +2519,28 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="B50" s="1" t="s">
+        <x:v>282</x:v>
+      </x:c>
+      <x:c r="C50" s="1" t="s">
+        <x:v>283</x:v>
+      </x:c>
+      <x:c r="D50" s="1" t="s">
+        <x:v>284</x:v>
+      </x:c>
+      <x:c r="E50" s="1" t="s">
+        <x:v>285</x:v>
+      </x:c>
+      <x:c r="F50" s="1" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G50" s="1" t="s">
         <x:v>286</x:v>
       </x:c>
-      <x:c r="C50" s="1" t="s">
-        <x:v>287</x:v>
-      </x:c>
-      <x:c r="D50" s="1" t="s">
-        <x:v>288</x:v>
-      </x:c>
-      <x:c r="E50" s="1" t="s">
-        <x:v>289</x:v>
-      </x:c>
-      <x:c r="F50" s="1" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G50" s="1" t="s">
-        <x:v>290</x:v>
-      </x:c>
       <x:c r="H50" s="1" t="s">
         <x:v>17</x:v>
       </x:c>
       <x:c r="I50" s="1" t="s">
-        <x:v>291</x:v>
+        <x:v>276</x:v>
       </x:c>
     </x:row>
     <x:row r="51" spans="1:9" ht="15" customHeight="1">
@@ -2560,28 +2548,28 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="B51" s="1" t="s">
+        <x:v>287</x:v>
+      </x:c>
+      <x:c r="C51" s="1" t="s">
+        <x:v>288</x:v>
+      </x:c>
+      <x:c r="D51" s="1" t="s">
+        <x:v>289</x:v>
+      </x:c>
+      <x:c r="E51" s="1" t="s">
+        <x:v>290</x:v>
+      </x:c>
+      <x:c r="F51" s="1" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G51" s="1" t="s">
+        <x:v>291</x:v>
+      </x:c>
+      <x:c r="H51" s="1" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I51" s="1" t="s">
         <x:v>292</x:v>
-      </x:c>
-      <x:c r="C51" s="1" t="s">
-        <x:v>293</x:v>
-      </x:c>
-      <x:c r="D51" s="1" t="s">
-        <x:v>294</x:v>
-      </x:c>
-      <x:c r="E51" s="1" t="s">
-        <x:v>295</x:v>
-      </x:c>
-      <x:c r="F51" s="1" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G51" s="1" t="s">
-        <x:v>296</x:v>
-      </x:c>
-      <x:c r="H51" s="1" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I51" s="1" t="s">
-        <x:v>291</x:v>
       </x:c>
     </x:row>
     <x:row r="52" spans="1:9" ht="15" customHeight="1">
@@ -2589,28 +2577,28 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="B52" s="1" t="s">
+        <x:v>293</x:v>
+      </x:c>
+      <x:c r="C52" s="1" t="s">
+        <x:v>294</x:v>
+      </x:c>
+      <x:c r="D52" s="1" t="s">
+        <x:v>295</x:v>
+      </x:c>
+      <x:c r="E52" s="1" t="s">
+        <x:v>296</x:v>
+      </x:c>
+      <x:c r="F52" s="1" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G52" s="1" t="s">
         <x:v>297</x:v>
       </x:c>
-      <x:c r="C52" s="1" t="s">
+      <x:c r="H52" s="1" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I52" s="1" t="s">
         <x:v>298</x:v>
-      </x:c>
-      <x:c r="D52" s="1" t="s">
-        <x:v>299</x:v>
-      </x:c>
-      <x:c r="E52" s="1" t="s">
-        <x:v>300</x:v>
-      </x:c>
-      <x:c r="F52" s="1" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G52" s="1" t="s">
-        <x:v>301</x:v>
-      </x:c>
-      <x:c r="H52" s="1" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I52" s="1" t="s">
-        <x:v>302</x:v>
       </x:c>
     </x:row>
     <x:row r="53" spans="1:9" ht="15" customHeight="1">
@@ -2618,28 +2606,28 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="B53" s="1" t="s">
+        <x:v>299</x:v>
+      </x:c>
+      <x:c r="C53" s="1" t="s">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="D53" s="1" t="s">
+        <x:v>301</x:v>
+      </x:c>
+      <x:c r="E53" s="1" t="s">
+        <x:v>302</x:v>
+      </x:c>
+      <x:c r="F53" s="1" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G53" s="1" t="s">
         <x:v>303</x:v>
       </x:c>
-      <x:c r="C53" s="1" t="s">
+      <x:c r="H53" s="1" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I53" s="1" t="s">
         <x:v>304</x:v>
-      </x:c>
-      <x:c r="D53" s="1" t="s">
-        <x:v>305</x:v>
-      </x:c>
-      <x:c r="E53" s="1" t="s">
-        <x:v>306</x:v>
-      </x:c>
-      <x:c r="F53" s="1" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G53" s="1" t="s">
-        <x:v>307</x:v>
-      </x:c>
-      <x:c r="H53" s="1" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I53" s="1" t="s">
-        <x:v>308</x:v>
       </x:c>
     </x:row>
     <x:row r="54" spans="1:9" ht="15" customHeight="1">
@@ -2647,28 +2635,28 @@
         <x:v>51</x:v>
       </x:c>
       <x:c r="B54" s="1" t="s">
+        <x:v>305</x:v>
+      </x:c>
+      <x:c r="C54" s="1" t="s">
+        <x:v>306</x:v>
+      </x:c>
+      <x:c r="D54" s="1" t="s">
+        <x:v>307</x:v>
+      </x:c>
+      <x:c r="E54" s="1" t="s">
+        <x:v>308</x:v>
+      </x:c>
+      <x:c r="F54" s="1" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G54" s="1" t="s">
         <x:v>309</x:v>
       </x:c>
-      <x:c r="C54" s="1" t="s">
-        <x:v>310</x:v>
-      </x:c>
-      <x:c r="D54" s="1" t="s">
-        <x:v>311</x:v>
-      </x:c>
-      <x:c r="E54" s="1" t="s">
-        <x:v>312</x:v>
-      </x:c>
-      <x:c r="F54" s="1" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G54" s="1" t="s">
-        <x:v>313</x:v>
-      </x:c>
       <x:c r="H54" s="1" t="s">
         <x:v>17</x:v>
       </x:c>
       <x:c r="I54" s="1" t="s">
-        <x:v>314</x:v>
+        <x:v>304</x:v>
       </x:c>
     </x:row>
     <x:row r="55" spans="1:9" ht="15" customHeight="1">
@@ -2676,28 +2664,28 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="B55" s="1" t="s">
+        <x:v>310</x:v>
+      </x:c>
+      <x:c r="C55" s="1" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D55" s="1" t="s">
+        <x:v>311</x:v>
+      </x:c>
+      <x:c r="E55" s="1" t="s">
+        <x:v>312</x:v>
+      </x:c>
+      <x:c r="F55" s="1" t="s">
+        <x:v>313</x:v>
+      </x:c>
+      <x:c r="G55" s="1" t="s">
+        <x:v>314</x:v>
+      </x:c>
+      <x:c r="H55" s="1" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I55" s="1" t="s">
         <x:v>315</x:v>
-      </x:c>
-      <x:c r="C55" s="1" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D55" s="1" t="s">
-        <x:v>316</x:v>
-      </x:c>
-      <x:c r="E55" s="1" t="s">
-        <x:v>317</x:v>
-      </x:c>
-      <x:c r="F55" s="1" t="s">
-        <x:v>318</x:v>
-      </x:c>
-      <x:c r="G55" s="1" t="s">
-        <x:v>319</x:v>
-      </x:c>
-      <x:c r="H55" s="1" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I55" s="1" t="s">
-        <x:v>320</x:v>
       </x:c>
     </x:row>
     <x:row r="56" spans="1:9" ht="15" customHeight="1">
@@ -2705,28 +2693,28 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="B56" s="1" t="s">
-        <x:v>321</x:v>
+        <x:v>316</x:v>
       </x:c>
       <x:c r="C56" s="1" t="s">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D56" s="1" t="s">
-        <x:v>316</x:v>
+        <x:v>311</x:v>
       </x:c>
       <x:c r="E56" s="1" t="s">
-        <x:v>322</x:v>
+        <x:v>317</x:v>
       </x:c>
       <x:c r="F56" s="1" t="s">
+        <x:v>313</x:v>
+      </x:c>
+      <x:c r="G56" s="1" t="s">
         <x:v>318</x:v>
       </x:c>
-      <x:c r="G56" s="1" t="s">
-        <x:v>323</x:v>
-      </x:c>
       <x:c r="H56" s="1" t="s">
         <x:v>17</x:v>
       </x:c>
       <x:c r="I56" s="1" t="s">
-        <x:v>320</x:v>
+        <x:v>319</x:v>
       </x:c>
     </x:row>
     <x:row r="57" spans="1:9" ht="15" customHeight="1">
@@ -2734,28 +2722,28 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="B57" s="1" t="s">
-        <x:v>324</x:v>
+        <x:v>320</x:v>
       </x:c>
       <x:c r="C57" s="1" t="s">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D57" s="1" t="s">
-        <x:v>316</x:v>
+        <x:v>311</x:v>
       </x:c>
       <x:c r="E57" s="1" t="s">
         <x:v>17</x:v>
       </x:c>
       <x:c r="F57" s="1" t="s">
+        <x:v>313</x:v>
+      </x:c>
+      <x:c r="G57" s="1" t="s">
         <x:v>318</x:v>
       </x:c>
-      <x:c r="G57" s="1" t="s">
-        <x:v>323</x:v>
-      </x:c>
       <x:c r="H57" s="1" t="s">
         <x:v>17</x:v>
       </x:c>
       <x:c r="I57" s="1" t="s">
-        <x:v>320</x:v>
+        <x:v>319</x:v>
       </x:c>
     </x:row>
     <x:row r="58" spans="1:9" ht="15" customHeight="1">
@@ -2763,28 +2751,28 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="B58" s="1" t="s">
-        <x:v>325</x:v>
+        <x:v>321</x:v>
       </x:c>
       <x:c r="C58" s="1" t="s">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D58" s="1" t="s">
-        <x:v>316</x:v>
+        <x:v>311</x:v>
       </x:c>
       <x:c r="E58" s="1" t="s">
         <x:v>17</x:v>
       </x:c>
       <x:c r="F58" s="1" t="s">
-        <x:v>318</x:v>
+        <x:v>313</x:v>
       </x:c>
       <x:c r="G58" s="1" t="s">
-        <x:v>326</x:v>
+        <x:v>322</x:v>
       </x:c>
       <x:c r="H58" s="1" t="s">
         <x:v>17</x:v>
       </x:c>
       <x:c r="I58" s="1" t="s">
-        <x:v>320</x:v>
+        <x:v>319</x:v>
       </x:c>
     </x:row>
     <x:row r="59" spans="1:9" ht="15" customHeight="1">
@@ -2792,28 +2780,28 @@
         <x:v>56</x:v>
       </x:c>
       <x:c r="B59" s="1" t="s">
-        <x:v>327</x:v>
+        <x:v>323</x:v>
       </x:c>
       <x:c r="C59" s="1" t="s">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D59" s="1" t="s">
-        <x:v>316</x:v>
+        <x:v>311</x:v>
       </x:c>
       <x:c r="E59" s="1" t="s">
-        <x:v>328</x:v>
+        <x:v>324</x:v>
       </x:c>
       <x:c r="F59" s="1" t="s">
-        <x:v>318</x:v>
+        <x:v>313</x:v>
       </x:c>
       <x:c r="G59" s="1" t="s">
-        <x:v>329</x:v>
+        <x:v>325</x:v>
       </x:c>
       <x:c r="H59" s="1" t="s">
         <x:v>17</x:v>
       </x:c>
       <x:c r="I59" s="1" t="s">
-        <x:v>320</x:v>
+        <x:v>319</x:v>
       </x:c>
     </x:row>
     <x:row r="60" spans="1:9" ht="15" customHeight="1">
@@ -2821,28 +2809,28 @@
         <x:v>57</x:v>
       </x:c>
       <x:c r="B60" s="1" t="s">
-        <x:v>330</x:v>
+        <x:v>326</x:v>
       </x:c>
       <x:c r="C60" s="1" t="s">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D60" s="1" t="s">
-        <x:v>316</x:v>
+        <x:v>311</x:v>
       </x:c>
       <x:c r="E60" s="1" t="s">
-        <x:v>331</x:v>
+        <x:v>327</x:v>
       </x:c>
       <x:c r="F60" s="1" t="s">
-        <x:v>318</x:v>
+        <x:v>313</x:v>
       </x:c>
       <x:c r="G60" s="1" t="s">
-        <x:v>332</x:v>
+        <x:v>328</x:v>
       </x:c>
       <x:c r="H60" s="1" t="s">
         <x:v>17</x:v>
       </x:c>
       <x:c r="I60" s="1" t="s">
-        <x:v>320</x:v>
+        <x:v>319</x:v>
       </x:c>
     </x:row>
     <x:row r="61" spans="1:9" ht="15" customHeight="1">
@@ -2853,7 +2841,7 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="C61" s="1" t="s">
-        <x:v>333</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="D61" s="1" t="s">
         <x:v>17</x:v>
@@ -2862,21 +2850,21 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="F61" s="1" t="s">
-        <x:v>334</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="G61" s="1" t="s">
-        <x:v>335</x:v>
+        <x:v>331</x:v>
       </x:c>
       <x:c r="H61" s="1" t="s">
         <x:v>17</x:v>
       </x:c>
       <x:c r="I61" s="1" t="s">
-        <x:v>336</x:v>
+        <x:v>332</x:v>
       </x:c>
     </x:row>
     <x:row r="62" spans="1:9" ht="15" customHeight="1">
       <x:c r="A62" s="2" t="s">
-        <x:v>337</x:v>
+        <x:v>333</x:v>
       </x:c>
       <x:c r="B62" s="2" t="s">
         <x:v>1</x:v>

</xml_diff>